<commit_message>
PAUSED (task137): round 2 redesign, stage 3 green, waiting on the reader and judge
The 10/10 audit's redesign: the decisive step moves from the repricing drop to the class of the money
(what a new-money special won, which goes to the retention offer at its first maturity whatever its drop,
against member money, which goes with the drop). Book 5,250 agent-hours (1,250, 2,000, 2,000); the share
by drop books 4,250, the audit's locked-rate-by-term logit 4,500, every one of 22 rivals two bins or more
under. Ask A's link moved into the payments narrative, Ask B's overlap into hand-moved certificates with
capitalised interest; the prompt's ask wording rewritten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task137/golden/td_booking_q1_2027.xlsx
+++ b/task137/golden/td_booking_q1_2027.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="68">
   <si>
     <t>TDR-2027Q1: agent-hours to book with Harbourline Contact Services</t>
   </si>
@@ -75,13 +75,13 @@
     <t>Do-not-call wash at the cut</t>
   </si>
   <si>
-    <t>460 deposits have no callable number once the holders' numbers are washed against the register as it stood on 2 November 2026; they are not released (procedure 4.3) and carry no hours.</t>
+    <t>464 deposits have no callable number once the holders' numbers are washed against the register as it stood on 2 November 2026; they are not released (procedure 4.3) and carry no hours.</t>
   </si>
   <si>
     <t>Release</t>
   </si>
   <si>
-    <t>95.5 per cent of listed deposits with a callable number reached release in the seven closed campaigns; the rest had given instructions first (procedure 4.2).</t>
+    <t>95.2 per cent of listed deposits with a callable number reached release in the seven closed campaigns; the rest had given instructions first (procedure 4.2).</t>
   </si>
   <si>
     <t>Dialling</t>
@@ -93,7 +93,7 @@
     <t>Retention offer</t>
   </si>
   <si>
-    <t>Each deposit's chance that a conversation goes to the retention offer is the share of past conversations at the same drop from the locked rate to the reinvestment rate for its term (0.25-point bands). The list's drops are read against the January to March 2027 rates in the campaign brief: 10,735 four-year deposits at 5.65 per cent meet the 3.15 per cent card, a drop of 2.50 points, where 92 per cent of past conversations went to the retention offer.</t>
+    <t>Each deposit's chance that a conversation goes to the retention offer is the share of past conversations of its class at the same drop from its rate to the reinvestment rate for its term (0.25-point bands). Money a special won (a rate 0.40 points or more above the lowest rate of the deposits of its term opened in the same quarter) went to the offer at 87 per cent of 4,093 conversations in the seven campaigns, much the same at every drop; other deposits far less often, more as the drop grows (28 per cent at drops of 1.50 to 1.75 points, where special money ran at 88). 10,697 4-year deposits opened at the 5.65 per cent special (the other 4-year deposits of January to March 2023 from 5.15 per cent) meet the 4.00 per cent rate for January to March 2027, a drop of 1.65 points.</t>
   </si>
   <si>
     <t>Minutes</t>
@@ -102,10 +102,10 @@
     <t>1.5 per dial that does not reach the holder, 8 per conversation, 22 per retention-offer conversation (schedule 2). Hours to book rounded to the nearest 250 (procedure 6.1).</t>
   </si>
   <si>
-    <t>Deposits on each closed campaign's list still on term deposit with the Society 30 days after maturity</t>
-  </si>
-  <si>
-    <t>Reinvested on the deposit's own account at maturity, or the maturity proceeds paid that day into a term deposit opened with them; either still open 30 days after maturity. Principal kept: the deposit's principal, or the proceeds transferred into the new deposit. NZ$, nearest thousand.</t>
+    <t>Principal on each closed campaign's list still on term deposit with the Society 30 days after maturity</t>
+  </si>
+  <si>
+    <t>Reinvested on the deposit's own account at maturity, or maturity proceeds paid for it that day into a term deposit opened with them; either still open 30 days after maturity. Principal: the deposit's own, or the proceeds paid into the new deposit (new money added to it excluded). NZ$, nearest thousand.</t>
   </si>
   <si>
     <t>Campaign</t>
@@ -114,12 +114,12 @@
     <t>Maturities</t>
   </si>
   <si>
-    <t>Still on term deposit at 30 days</t>
-  </si>
-  <si>
     <t>Principal still on term deposit (NZ$)</t>
   </si>
   <si>
+    <t>Deposits it came from</t>
+  </si>
+  <si>
     <t>TDR-2025Q1</t>
   </si>
   <si>
@@ -165,13 +165,16 @@
     <t>Principal maturing January to March 2027: term deposits and investment certificates, all members</t>
   </si>
   <si>
-    <t>Term deposits and certificates held in the core on 2 November 2026, each account once, and the certificates still on the investment platform; the part not on the TDR-2027Q1 list. NZ$, nearest thousand.</t>
+    <t>Term deposits and certificates held in the core on 2 November 2026, each account once, and the certificates still on the investment platform; the quarter's part not on the TDR-2027Q1 list. NZ$, nearest thousand.</t>
   </si>
   <si>
     <t>Principal maturing (NZ$)</t>
   </si>
   <si>
-    <t>Not on the list (NZ$)</t>
+    <t>Not on the list</t>
+  </si>
+  <si>
+    <t>the quarter's maturing principal less the list's</t>
   </si>
   <si>
     <t>Notes</t>
@@ -195,7 +198,13 @@
     <t>Drop</t>
   </si>
   <si>
-    <t>The deposit's rate less the reinvestment rate for its term in the campaign brief for the quarter it matures in. Shares of past conversations are taken in 0.25-point bands of drop across all seven closed campaigns, as procedure 6.1 has the forecast draw on every closed campaign.</t>
+    <t>The deposit's rate less the reinvestment rate for its term in the campaign brief for the quarter it matures in. Shares of past conversations are taken by class in 0.25-point bands of drop across all seven closed campaigns, as procedure 6.1 has the forecast draw on every closed campaign.</t>
+  </si>
+  <si>
+    <t>Special money</t>
+  </si>
+  <si>
+    <t>A deposit whose rate is 0.40 points or more above the lowest rate among the same list's deposits of its term opened in the same quarter (the specials sold new money one rate for every amount; other deposits sit on the posted rate or up to 0.25 above it). In the seven campaigns: the one-year deposits at 6.35, 5.45, 5.10, 4.75 and 4.45 per cent, the two-year at 6.30 and the three-year at 6.00.</t>
   </si>
   <si>
     <t>Not released</t>
@@ -213,13 +222,13 @@
     <t>Kept at 30 days</t>
   </si>
   <si>
-    <t>Own-account reinvestments, and maturity proceeds paid that day into a new term deposit, still open 30 days after maturity; new money added to a new deposit is not counted.</t>
+    <t>Own-account reinvestments, and maturity proceeds the payments system paid for the deposit that day into a new term deposit (its settlement payments name the matured account in the narrative), still open 30 days after maturity; new money added to a new deposit is not counted.</t>
   </si>
   <si>
     <t>Maturing Q1 2027</t>
   </si>
   <si>
-    <t>The core holdings view lists a joint deposit under each holder; counted once per account. Certificates still on the investment platform are taken from its register of 30 June 2026, less those the migration batches moved to the core.</t>
+    <t>The core holdings view lists a joint deposit under each holder; counted once per account, at the core's principal. Certificates still on the investment platform are taken from its register of 30 June 2026, less those already in the core: moved by a migration batch, or moved by hand and found by issue date, maturity date, rate and term.</t>
   </si>
 </sst>
 </file>
@@ -318,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -342,6 +351,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -704,25 +714,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4">
-        <v>5030</v>
+        <v>4474</v>
       </c>
       <c r="C5" s="4">
-        <v>4902</v>
+        <v>4354</v>
       </c>
       <c r="D5" s="4">
-        <v>18383</v>
+        <v>16160</v>
       </c>
       <c r="E5" s="4">
-        <v>3799</v>
+        <v>3379</v>
       </c>
       <c r="F5" s="4">
-        <v>2201</v>
+        <v>1510</v>
       </c>
       <c r="G5" s="5">
-        <v>1479.5</v>
+        <v>1206.9</v>
       </c>
       <c r="H5" s="6">
-        <v>1500</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -730,22 +740,22 @@
         <v>11</v>
       </c>
       <c r="B6" s="4">
-        <v>6631</v>
+        <v>6835</v>
       </c>
       <c r="C6" s="4">
-        <v>6476</v>
+        <v>6666</v>
       </c>
       <c r="D6" s="4">
-        <v>24238</v>
+        <v>24747</v>
       </c>
       <c r="E6" s="4">
-        <v>5034</v>
+        <v>5184</v>
       </c>
       <c r="F6" s="4">
-        <v>3287</v>
+        <v>3014</v>
       </c>
       <c r="G6" s="5">
-        <v>2044.1</v>
+        <v>2013.3</v>
       </c>
       <c r="H6" s="6">
         <v>2000</v>
@@ -756,22 +766,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="4">
-        <v>6739</v>
+        <v>7091</v>
       </c>
       <c r="C7" s="4">
-        <v>6562</v>
+        <v>6916</v>
       </c>
       <c r="D7" s="4">
-        <v>24735</v>
+        <v>25808</v>
       </c>
       <c r="E7" s="4">
-        <v>5126</v>
+        <v>5399</v>
       </c>
       <c r="F7" s="4">
-        <v>3182</v>
+        <v>2982</v>
       </c>
       <c r="G7" s="5">
-        <v>2044.4</v>
+        <v>2060.7</v>
       </c>
       <c r="H7" s="6">
         <v>2000</v>
@@ -785,22 +795,22 @@
         <v>18400</v>
       </c>
       <c r="C8" s="7">
-        <v>17940</v>
+        <v>17936</v>
       </c>
       <c r="D8" s="7">
-        <v>67355</v>
+        <v>66715</v>
       </c>
       <c r="E8" s="7">
-        <v>13959</v>
+        <v>13962</v>
       </c>
       <c r="F8" s="7">
-        <v>8670</v>
+        <v>7506</v>
       </c>
       <c r="G8" s="8">
-        <v>5568</v>
+        <v>5280.9</v>
       </c>
       <c r="H8" s="9">
-        <v>5500</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -832,7 +842,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="56" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>21</v>
       </c>
@@ -872,8 +882,8 @@
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -914,10 +924,10 @@
         <v>7612</v>
       </c>
       <c r="D5" s="4">
-        <v>6520</v>
+        <v>497825000</v>
       </c>
       <c r="E5" s="4">
-        <v>486794000</v>
+        <v>6700</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -928,13 +938,13 @@
         <v>34</v>
       </c>
       <c r="C6" s="4">
-        <v>8724</v>
+        <v>8651</v>
       </c>
       <c r="D6" s="4">
-        <v>7007</v>
+        <v>537491000</v>
       </c>
       <c r="E6" s="4">
-        <v>526875000</v>
+        <v>7186</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -945,13 +955,13 @@
         <v>36</v>
       </c>
       <c r="C7" s="4">
-        <v>8607</v>
+        <v>8567</v>
       </c>
       <c r="D7" s="4">
-        <v>6902</v>
+        <v>532430000</v>
       </c>
       <c r="E7" s="4">
-        <v>504704000</v>
+        <v>7226</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -962,13 +972,13 @@
         <v>38</v>
       </c>
       <c r="C8" s="4">
-        <v>8658</v>
+        <v>8705</v>
       </c>
       <c r="D8" s="4">
-        <v>6917</v>
+        <v>536002000</v>
       </c>
       <c r="E8" s="4">
-        <v>500989000</v>
+        <v>7172</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -979,13 +989,13 @@
         <v>40</v>
       </c>
       <c r="C9" s="4">
-        <v>8494</v>
+        <v>9010</v>
       </c>
       <c r="D9" s="4">
-        <v>6860</v>
+        <v>562096000</v>
       </c>
       <c r="E9" s="4">
-        <v>503624000</v>
+        <v>7591</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -996,13 +1006,13 @@
         <v>42</v>
       </c>
       <c r="C10" s="4">
-        <v>8502</v>
+        <v>8970</v>
       </c>
       <c r="D10" s="4">
-        <v>6933</v>
+        <v>557067000</v>
       </c>
       <c r="E10" s="4">
-        <v>512433000</v>
+        <v>7494</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1013,13 +1023,13 @@
         <v>44</v>
       </c>
       <c r="C11" s="4">
-        <v>8668</v>
+        <v>9240</v>
       </c>
       <c r="D11" s="4">
-        <v>7001</v>
+        <v>573831000</v>
       </c>
       <c r="E11" s="4">
-        <v>521207000</v>
+        <v>7765</v>
       </c>
     </row>
   </sheetData>
@@ -1036,12 +1046,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1061,19 +1071,13 @@
       <c r="B4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>48</v>
-      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="4">
-        <v>467102000</v>
-      </c>
-      <c r="C5" s="4">
-        <v>60860000</v>
+        <v>415506000</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1081,10 +1085,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="4">
-        <v>633665000</v>
-      </c>
-      <c r="C6" s="4">
-        <v>74665000</v>
+        <v>646816000</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1092,10 +1093,26 @@
         <v>12</v>
       </c>
       <c r="B7" s="4">
-        <v>633034000</v>
-      </c>
-      <c r="C7" s="4">
-        <v>80661000</v>
+        <v>672944000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="7">
+        <v>1735266000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="6">
+        <v>214491000</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1112,7 +1129,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -1121,71 +1138,79 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>50</v>
+      <c r="A3" s="16" t="s">
+        <v>51</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
-        <v>52</v>
+      <c r="A4" s="16" t="s">
+        <v>53</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>21</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
         <v>55</v>
       </c>
+    </row>
+    <row r="6" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>56</v>
+      </c>
       <c r="B6" s="12" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
         <v>57</v>
       </c>
+    </row>
+    <row r="7" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="B7" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
-        <v>59</v>
+      <c r="A8" s="16" t="s">
+        <v>60</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
-        <v>61</v>
+      <c r="A9" s="16" t="s">
+        <v>62</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
-        <v>63</v>
+      <c r="A10" s="16" t="s">
+        <v>64</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>